<commit_message>
Added new scene over weekend
Nothing changed to the copied scene, but I plan to actually make the game there.
</commit_message>
<xml_diff>
--- a/TestPlanTemplate.xlsx
+++ b/TestPlanTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UnityZakFMP\FMP-Concepts\FMP-Concepts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ZakUnityFMP\FMP-Concepts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4379F0C-25C1-4128-A875-D7690373C89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{422A1EFC-0C5C-4E0B-B4AD-4BA26E2D17D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="166" xr2:uid="{D9B1ECAE-43F8-4EE8-A9A6-870A8BC1A0C0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="166" xr2:uid="{D9B1ECAE-43F8-4EE8-A9A6-870A8BC1A0C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="57">
   <si>
     <t>Test Number</t>
   </si>
@@ -176,6 +176,60 @@
   </si>
   <si>
     <t>BasicEnemyAIBehaviour Scene</t>
+  </si>
+  <si>
+    <t>01.05.26</t>
+  </si>
+  <si>
+    <t>Moving the player</t>
+  </si>
+  <si>
+    <t>PlayerBehavior in HarrisonFerrone chapters</t>
+  </si>
+  <si>
+    <t>trying to read Input using the UnityEngine.Input class, but you have switched active Input handling to Input System package in Player Settings</t>
+  </si>
+  <si>
+    <t>Said error goes after switching to "both" from "Input system Package(new)"</t>
+  </si>
+  <si>
+    <t>The error dissapeared</t>
+  </si>
+  <si>
+    <t>Found solution thanks to this post on https://discussions.unity.com/t/help-me-how-to-fix-it/813420 by lawrenceblasco7812.</t>
+  </si>
+  <si>
+    <t>A / D cause player rotate left and right vertically</t>
+  </si>
+  <si>
+    <t>player rotates horizontally(so you can turn)</t>
+  </si>
+  <si>
+    <t>Player now rotates horizontally</t>
+  </si>
+  <si>
+    <t>On line "this.transform.Rotate(Vector3.up * hInput * Time.deltaTime);" I wrote Vector3.forward instead of Vector3.up.</t>
+  </si>
+  <si>
+    <t>02.05.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bullets disapear after </t>
+  </si>
+  <si>
+    <t>bulletBehavior in HarrisonFerrone chapters</t>
+  </si>
+  <si>
+    <t>Left click creates a bullet -&gt; wants to disapear after 3 seconds</t>
+  </si>
+  <si>
+    <t>After 3 seconds the bullet disapears</t>
+  </si>
+  <si>
+    <t>Bullets do disapear</t>
+  </si>
+  <si>
+    <t>Forgot to add rigidbody</t>
   </si>
 </sst>
 </file>
@@ -626,7 +680,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{578B1A4F-6B1D-4B59-8AFF-2D563D27525C}">
   <dimension ref="A1:H101"/>
-  <sheetFormatPr defaultRowHeight="23.25" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="24" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="3"/>
     <col min="2" max="2" width="15.6640625" style="4" customWidth="1"/>
@@ -639,7 +693,7 @@
     <col min="9" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="36" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -665,7 +719,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -689,7 +743,7 @@
       </c>
       <c r="H2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="48" x14ac:dyDescent="0.4">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -715,7 +769,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="48" x14ac:dyDescent="0.4">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -738,7 +792,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -761,7 +815,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="48" x14ac:dyDescent="0.4">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -781,7 +835,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="48" x14ac:dyDescent="0.4">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -804,7 +858,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" ht="48" x14ac:dyDescent="0.4">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -827,7 +881,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -842,553 +896,613 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="72" x14ac:dyDescent="0.4">
       <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="F11" s="4"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="48" x14ac:dyDescent="0.4">
       <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="F12" s="4"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B12" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13" s="3">
         <v>12</v>
       </c>
       <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H13" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14" s="3">
         <v>13</v>
       </c>
       <c r="F14" s="4"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A15" s="3">
         <v>14</v>
       </c>
       <c r="F15" s="4"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A16" s="3">
         <v>15</v>
       </c>
       <c r="F16" s="4"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17" s="3">
         <v>16</v>
       </c>
       <c r="F17" s="4"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18" s="3">
         <v>17</v>
       </c>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19" s="3">
         <v>18</v>
       </c>
       <c r="F19" s="4"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" s="3">
         <v>19</v>
       </c>
       <c r="F20" s="4"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22" s="3">
         <v>21</v>
       </c>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23" s="3">
         <v>22</v>
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25" s="3">
         <v>24</v>
       </c>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26" s="3">
         <v>25</v>
       </c>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27" s="3">
         <v>26</v>
       </c>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28" s="3">
         <v>27</v>
       </c>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29" s="3">
         <v>28</v>
       </c>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30" s="3">
         <v>29</v>
       </c>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31" s="3">
         <v>30</v>
       </c>
       <c r="F31" s="4"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32" s="3">
         <v>31</v>
       </c>
       <c r="F32" s="4"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33" s="3">
         <v>32</v>
       </c>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A34" s="3">
         <v>33</v>
       </c>
       <c r="F34" s="4"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A35" s="3">
         <v>34</v>
       </c>
       <c r="F35" s="4"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A36" s="3">
         <v>35</v>
       </c>
       <c r="F36" s="4"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A37" s="3">
         <v>36</v>
       </c>
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A38" s="3">
         <v>37</v>
       </c>
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39" s="3">
         <v>38</v>
       </c>
       <c r="F39" s="4"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40" s="3">
         <v>39</v>
       </c>
       <c r="F40" s="4"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41" s="3">
         <v>40</v>
       </c>
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="F42" s="4"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43" s="3">
         <v>42</v>
       </c>
       <c r="F43" s="4"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44" s="3">
         <v>43</v>
       </c>
       <c r="F44" s="4"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45" s="3">
         <v>44</v>
       </c>
       <c r="F45" s="4"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A46" s="3">
         <v>45</v>
       </c>
       <c r="F46" s="4"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A47" s="3">
         <v>46</v>
       </c>
       <c r="F47" s="4"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A48" s="3">
         <v>47</v>
       </c>
       <c r="F48" s="4"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A49" s="3">
         <v>48</v>
       </c>
       <c r="F49" s="4"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A50" s="3">
         <v>49</v>
       </c>
       <c r="F50" s="4"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A51" s="3">
         <v>50</v>
       </c>
       <c r="F51" s="4"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A52" s="3">
         <v>51</v>
       </c>
       <c r="F52" s="4"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A53" s="3">
         <v>52</v>
       </c>
       <c r="F53" s="4"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A54" s="3">
         <v>53</v>
       </c>
       <c r="F54" s="4"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A55" s="3">
         <v>54</v>
       </c>
       <c r="F55" s="4"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A56" s="3">
         <v>55</v>
       </c>
       <c r="F56" s="4"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A57" s="3">
         <v>56</v>
       </c>
       <c r="F57" s="4"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A58" s="3">
         <v>57</v>
       </c>
       <c r="F58" s="4"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A59" s="3">
         <v>58</v>
       </c>
       <c r="F59" s="4"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A60" s="3">
         <v>59</v>
       </c>
       <c r="F60" s="4"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A61" s="3">
         <v>60</v>
       </c>
       <c r="F61" s="4"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A62" s="3">
         <v>61</v>
       </c>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A63" s="3">
         <v>62</v>
       </c>
       <c r="F63" s="4"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A64" s="3">
         <v>63</v>
       </c>
       <c r="F64" s="4"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A65" s="3">
         <v>64</v>
       </c>
       <c r="F65" s="4"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A66" s="3">
         <v>65</v>
       </c>
       <c r="F66" s="4"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A67" s="3">
         <v>66</v>
       </c>
       <c r="F67" s="4"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A68" s="3">
         <v>67</v>
       </c>
       <c r="F68" s="4"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A69" s="3">
         <v>68</v>
       </c>
       <c r="F69" s="4"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A70" s="3">
         <v>69</v>
       </c>
       <c r="F70" s="4"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A71" s="3">
         <v>70</v>
       </c>
       <c r="F71" s="4"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A72" s="3">
         <v>71</v>
       </c>
       <c r="F72" s="4"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A73" s="3">
         <v>72</v>
       </c>
       <c r="F73" s="4"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A74" s="3">
         <v>73</v>
       </c>
       <c r="F74" s="4"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A75" s="3">
         <v>74</v>
       </c>
       <c r="F75" s="4"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A76" s="3">
         <v>75</v>
       </c>
       <c r="F76" s="4"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A77" s="3">
         <v>76</v>
       </c>
       <c r="F77" s="4"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A78" s="3">
         <v>77</v>
       </c>
       <c r="F78" s="4"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A79" s="3">
         <v>78</v>
       </c>
       <c r="F79" s="4"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A80" s="3">
         <v>79</v>
       </c>
       <c r="F80" s="4"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A81" s="3">
         <v>80</v>
       </c>
       <c r="F81" s="4"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A82" s="3">
         <v>81</v>
       </c>
       <c r="F82" s="4"/>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="F83" s="4"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="F84" s="4"/>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A85" s="3">
         <v>84</v>
       </c>
       <c r="F85" s="4"/>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A86" s="3">
         <v>85</v>
       </c>
       <c r="F86" s="4"/>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A87" s="3">
         <v>86</v>
       </c>
       <c r="F87" s="4"/>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A88" s="3">
         <v>87</v>
       </c>
       <c r="F88" s="4"/>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A89" s="3">
         <v>88</v>
       </c>
       <c r="F89" s="4"/>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A90" s="3">
         <v>89</v>
       </c>
       <c r="F90" s="4"/>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A91" s="3">
         <v>90</v>
       </c>
       <c r="F91" s="4"/>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A92" s="3">
         <v>91</v>
       </c>
       <c r="F92" s="4"/>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A93" s="3">
         <v>92</v>
       </c>
       <c r="F93" s="4"/>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A94" s="3">
         <v>93</v>
       </c>
       <c r="F94" s="4"/>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A95" s="3">
         <v>94</v>
       </c>
       <c r="F95" s="4"/>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A96" s="3">
         <v>95</v>
       </c>
       <c r="F96" s="4"/>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A97" s="3">
         <v>96</v>
       </c>
       <c r="F97" s="4"/>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A98" s="3">
         <v>97</v>
       </c>
       <c r="F98" s="4"/>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A99" s="3">
         <v>98</v>
       </c>
       <c r="F99" s="4"/>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A100" s="3">
         <v>99</v>
       </c>
       <c r="F100" s="4"/>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.4">
       <c r="F101" s="4"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated test log + miscellaneous
</commit_message>
<xml_diff>
--- a/TestPlanTemplate.xlsx
+++ b/TestPlanTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ZakUnityFMP\FMP Concepts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC926ED4-115E-451D-8188-04F0FCBC7892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED367A1-BAB9-4C20-8007-3D4150E7644E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="166" xr2:uid="{D9B1ECAE-43F8-4EE8-A9A6-870A8BC1A0C0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="106">
   <si>
     <t>Test Number</t>
   </si>
@@ -309,12 +309,81 @@
   <si>
     <t>Marked yellow as even though it seems to be solved, this is the first time its happened and I can't take the time out to recreate and find the root causing the issue.</t>
   </si>
+  <si>
+    <t>06.05.26</t>
+  </si>
+  <si>
+    <t>using Unity.ProjectAuditor.Editor; added to script</t>
+  </si>
+  <si>
+    <t>Hopefully moves</t>
+  </si>
+  <si>
+    <t>Didn’t move still</t>
+  </si>
+  <si>
+    <t>Suggested by Mathew.</t>
+  </si>
+  <si>
+    <t>EnemyBehaviour.cs(HarrisonFerrone chapters)</t>
+  </si>
+  <si>
+    <t>Re-did script from previous step</t>
+  </si>
+  <si>
+    <t>Getting enemy to patrol to 1st location</t>
+  </si>
+  <si>
+    <t>The enemy will move to 1st point</t>
+  </si>
+  <si>
+    <t>Enemy does move to 1st patrol location</t>
+  </si>
+  <si>
+    <t>Asssuming the issue preventing me from progressing was this('int'... no definition for 'position' &amp; no accessible extention method 'position accepting first agrument of type 'int' found). Marked green but not certain as to what caused the issue. Also prevented me from adding script to enemy, which I hadn't done and didn't realise. Suggested by mathew.</t>
+  </si>
+  <si>
+    <t>Getting enemy to patrol all locations</t>
+  </si>
+  <si>
+    <t>EnemyBehavior.cs(HarrisonFerrone chapters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operator '%' cannot be applied to operands of type 'Transform' and 'int' </t>
+  </si>
+  <si>
+    <t>Issue resolves and enemy patrols the four points</t>
+  </si>
+  <si>
+    <t>Solved error.</t>
+  </si>
+  <si>
+    <t>I was meant to write "_LocationIndex = (_LocationIndex + 1) % Locations.Count;" but wrote "_agent.destination = Locations[_LocationIndex] % Locations.Count;" thinking of the previous line of code as of typing.</t>
+  </si>
+  <si>
+    <t>Writing player health code causing errors</t>
+  </si>
+  <si>
+    <t>GameBehavior.cs(HarrisonFerrone chapters)</t>
+  </si>
+  <si>
+    <t>Added "private Rigidbody _rb;" &amp; "private CapsuleCollider _col"</t>
+  </si>
+  <si>
+    <t>Adding the two lines should get rid of the errors if what I was told by Co pilot is the case</t>
+  </si>
+  <si>
+    <t>The issue is solved and errors have gone.</t>
+  </si>
+  <si>
+    <t>Done with aid from Co-pilot, had asked it about the issue and it mentioned about "needing to delcare" or something along those lines first(which I'm taking is what I've done here)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="18"/>
       <color theme="1"/>
@@ -361,8 +430,14 @@
       <name val="Figtree"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF9C0006"/>
+      <name val="Figtree"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -391,6 +466,11 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -416,12 +496,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -453,8 +534,12 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
+    <cellStyle name="Bad" xfId="3" builtinId="27"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -945,7 +1030,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:8" ht="33.75" x14ac:dyDescent="0.4">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -961,14 +1046,14 @@
       <c r="F7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="11" t="s">
         <v>30</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" ht="33.75" x14ac:dyDescent="0.4">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -984,7 +1069,7 @@
       <c r="F8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="11" t="s">
         <v>35</v>
       </c>
       <c r="H8" s="2" t="s">
@@ -1051,7 +1136,7 @@
       <c r="F11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="9" t="s">
         <v>48</v>
       </c>
       <c r="H11" s="4" t="s">
@@ -1077,7 +1162,7 @@
       <c r="F12" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="9" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1100,7 +1185,7 @@
       <c r="F13" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" s="11" t="s">
         <v>60</v>
       </c>
       <c r="H13" s="2" t="s">
@@ -1126,7 +1211,7 @@
       <c r="F14" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="11" t="s">
         <v>62</v>
       </c>
       <c r="H14" s="2" t="s">
@@ -1152,7 +1237,7 @@
       <c r="F15" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="11" t="s">
         <v>64</v>
       </c>
       <c r="H15" s="2" t="s">
@@ -1178,7 +1263,7 @@
       <c r="F16" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="11" t="s">
         <v>66</v>
       </c>
       <c r="H16" s="2" t="s">
@@ -1270,41 +1355,109 @@
       <c r="B20" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="C20" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="72" x14ac:dyDescent="0.4">
       <c r="A21" s="3">
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F21" s="4"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="48" x14ac:dyDescent="0.4">
       <c r="A22" s="3">
         <v>21</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F22" s="4"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="48" x14ac:dyDescent="0.4">
       <c r="A23" s="3">
         <v>22</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F23" s="4"/>
+        <v>83</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A24" s="3">
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>56</v>
+        <v>83</v>
       </c>
       <c r="F24" s="4"/>
     </row>

</xml_diff>

<commit_message>
Tried to add a platform
Wanted to have a moving platform so found a video tutorial. Got it mostly done but said platform doesn't move. Would try and figure it out but not at this time currently(23:00).
</commit_message>
<xml_diff>
--- a/TestPlanTemplate.xlsx
+++ b/TestPlanTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ZakUnityFMP\FMP Concepts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ZakUnityFMP\FMP-Concepts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C00B097C-8710-467D-83A7-433E1F0133EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6AEDFF9-3056-4F0B-BA74-3ED9817E67C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="166" xr2:uid="{D9B1ECAE-43F8-4EE8-A9A6-870A8BC1A0C0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="166" xr2:uid="{D9B1ECAE-43F8-4EE8-A9A6-870A8BC1A0C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="147">
   <si>
     <t>Test Number</t>
   </si>
@@ -546,12 +546,33 @@
   <si>
     <t xml:space="preserve">error CS0103: The name 'SetCountText' does not exist in the current context </t>
   </si>
+  <si>
+    <t>Moving platform</t>
+  </si>
+  <si>
+    <t>error CS1026: ) expected</t>
+  </si>
+  <si>
+    <t>Looked, found missing dot between other &amp; tag so adding should fix it</t>
+  </si>
+  <si>
+    <t>Collider' not contain definition for 'Transform' and no accessible extension method 'Transform' accepting a first argument of type 'Collider' could be found</t>
+  </si>
+  <si>
+    <t>'Collider' not contain definition for 'Transform' and no accessible extension method 'Transform' accepting a first argument of type 'Collider' could be found</t>
+  </si>
+  <si>
+    <t>transform references the transform property in Inspector, which is lowercase and so should fix the errors when changing the T to t on each line.</t>
+  </si>
+  <si>
+    <t>Platform not moving</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="18"/>
       <color theme="1"/>
@@ -670,7 +691,7 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -715,6 +736,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1062,7 +1086,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{578B1A4F-6B1D-4B59-8AFF-2D563D27525C}">
   <dimension ref="A1:H101"/>
-  <sheetFormatPr defaultRowHeight="24" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="24"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="3"/>
     <col min="2" max="2" width="15.6640625" style="4" customWidth="1"/>
@@ -1075,7 +1099,7 @@
     <col min="9" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="36" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" ht="36">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1101,7 +1125,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1125,7 +1149,7 @@
       </c>
       <c r="H2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="48">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1151,7 +1175,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" ht="48">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1174,7 +1198,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1197,7 +1221,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" ht="48">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1217,7 +1241,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="33.75" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:8" ht="33">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1240,7 +1264,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="33.75" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" ht="33">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1263,7 +1287,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:8">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1278,7 +1302,7 @@
       </c>
       <c r="G9" s="4"/>
     </row>
-    <row r="10" spans="1:8" ht="72" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:8" ht="72">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1304,7 +1328,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:8">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1330,7 +1354,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:8" ht="48">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1353,7 +1377,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:8">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1379,7 +1403,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:8">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1405,7 +1429,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:8">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1431,7 +1455,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:8">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1457,7 +1481,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:8" ht="48">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1483,7 +1507,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:8" ht="48">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1509,7 +1533,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:8" ht="48">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1535,7 +1559,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:8">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1561,7 +1585,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="72" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:8" ht="72">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1587,7 +1611,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:8" ht="48">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1613,7 +1637,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:8" ht="48">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1639,7 +1663,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="72" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:8" ht="72">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1665,7 +1689,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:8">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1691,7 +1715,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:8">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1712,7 +1736,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:8">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1738,12 +1762,12 @@
         <v>124</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:8" ht="48">
       <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>104</v>
+      <c r="B28" s="12">
+        <v>46153</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>120</v>
@@ -1764,12 +1788,12 @@
         <v>127</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:8" ht="48">
       <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>104</v>
+      <c r="B29" s="12">
+        <v>46153</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>120</v>
@@ -1790,12 +1814,12 @@
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:8" ht="48">
       <c r="A30" s="3">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>104</v>
+      <c r="B30" s="12">
+        <v>46153</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>120</v>
@@ -1816,10 +1840,13 @@
         <v>136</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:8" ht="48">
       <c r="A31" s="3">
         <v>30</v>
       </c>
+      <c r="B31" s="12">
+        <v>46153</v>
+      </c>
       <c r="C31" s="4" t="s">
         <v>120</v>
       </c>
@@ -1836,10 +1863,13 @@
         <v>135</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="48" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:8" ht="48">
       <c r="A32" s="3">
         <v>31</v>
       </c>
+      <c r="B32" s="12">
+        <v>46153</v>
+      </c>
       <c r="C32" s="4" t="s">
         <v>120</v>
       </c>
@@ -1851,421 +1881,461 @@
       </c>
       <c r="F32" s="4"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:8" ht="48">
       <c r="A33" s="3">
         <v>32</v>
       </c>
+      <c r="B33" s="12">
+        <v>46154</v>
+      </c>
       <c r="C33" s="4" t="s">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="F33" s="4"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="E33" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="72">
       <c r="A34" s="3">
         <v>33</v>
       </c>
-      <c r="F34" s="4"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B34" s="12">
+        <v>46154</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" s="3">
         <v>34</v>
       </c>
+      <c r="B35" s="12">
+        <v>46154</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>146</v>
+      </c>
       <c r="F35" s="4"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:8">
       <c r="A36" s="3">
         <v>35</v>
       </c>
       <c r="F36" s="4"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:8">
       <c r="A37" s="3">
         <v>36</v>
       </c>
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:8">
       <c r="A38" s="3">
         <v>37</v>
       </c>
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:8">
       <c r="A39" s="3">
         <v>38</v>
       </c>
       <c r="F39" s="4"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:8">
       <c r="A40" s="3">
         <v>39</v>
       </c>
       <c r="F40" s="4"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:8">
       <c r="A41" s="3">
         <v>40</v>
       </c>
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:8">
       <c r="A42" s="3">
         <v>41</v>
       </c>
       <c r="F42" s="4"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:8">
       <c r="A43" s="3">
         <v>42</v>
       </c>
       <c r="F43" s="4"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:8">
       <c r="A44" s="3">
         <v>43</v>
       </c>
       <c r="F44" s="4"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:8">
       <c r="A45" s="3">
         <v>44</v>
       </c>
       <c r="F45" s="4"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:8">
       <c r="A46" s="3">
         <v>45</v>
       </c>
       <c r="F46" s="4"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:8">
       <c r="A47" s="3">
         <v>46</v>
       </c>
       <c r="F47" s="4"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:8">
       <c r="A48" s="3">
         <v>47</v>
       </c>
       <c r="F48" s="4"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:6">
       <c r="A49" s="3">
         <v>48</v>
       </c>
       <c r="F49" s="4"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:6">
       <c r="A50" s="3">
         <v>49</v>
       </c>
       <c r="F50" s="4"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:6">
       <c r="A51" s="3">
         <v>50</v>
       </c>
       <c r="F51" s="4"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:6">
       <c r="A52" s="3">
         <v>51</v>
       </c>
       <c r="F52" s="4"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:6">
       <c r="A53" s="3">
         <v>52</v>
       </c>
       <c r="F53" s="4"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:6">
       <c r="A54" s="3">
         <v>53</v>
       </c>
       <c r="F54" s="4"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:6">
       <c r="A55" s="3">
         <v>54</v>
       </c>
       <c r="F55" s="4"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:6">
       <c r="A56" s="3">
         <v>55</v>
       </c>
       <c r="F56" s="4"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:6">
       <c r="A57" s="3">
         <v>56</v>
       </c>
       <c r="F57" s="4"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:6">
       <c r="A58" s="3">
         <v>57</v>
       </c>
       <c r="F58" s="4"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:6">
       <c r="A59" s="3">
         <v>58</v>
       </c>
       <c r="F59" s="4"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:6">
       <c r="A60" s="3">
         <v>59</v>
       </c>
       <c r="F60" s="4"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:6">
       <c r="A61" s="3">
         <v>60</v>
       </c>
       <c r="F61" s="4"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:6">
       <c r="A62" s="3">
         <v>61</v>
       </c>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:6">
       <c r="A63" s="3">
         <v>62</v>
       </c>
       <c r="F63" s="4"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:6">
       <c r="A64" s="3">
         <v>63</v>
       </c>
       <c r="F64" s="4"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:6">
       <c r="A65" s="3">
         <v>64</v>
       </c>
       <c r="F65" s="4"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:6">
       <c r="A66" s="3">
         <v>65</v>
       </c>
       <c r="F66" s="4"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:6">
       <c r="A67" s="3">
         <v>66</v>
       </c>
       <c r="F67" s="4"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:6">
       <c r="A68" s="3">
         <v>67</v>
       </c>
       <c r="F68" s="4"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:6">
       <c r="A69" s="3">
         <v>68</v>
       </c>
       <c r="F69" s="4"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:6">
       <c r="A70" s="3">
         <v>69</v>
       </c>
       <c r="F70" s="4"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:6">
       <c r="A71" s="3">
         <v>70</v>
       </c>
       <c r="F71" s="4"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:6">
       <c r="A72" s="3">
         <v>71</v>
       </c>
       <c r="F72" s="4"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:6">
       <c r="A73" s="3">
         <v>72</v>
       </c>
       <c r="F73" s="4"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:6">
       <c r="A74" s="3">
         <v>73</v>
       </c>
       <c r="F74" s="4"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:6">
       <c r="A75" s="3">
         <v>74</v>
       </c>
       <c r="F75" s="4"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:6">
       <c r="A76" s="3">
         <v>75</v>
       </c>
       <c r="F76" s="4"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:6">
       <c r="A77" s="3">
         <v>76</v>
       </c>
       <c r="F77" s="4"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:6">
       <c r="A78" s="3">
         <v>77</v>
       </c>
       <c r="F78" s="4"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:6">
       <c r="A79" s="3">
         <v>78</v>
       </c>
       <c r="F79" s="4"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:6">
       <c r="A80" s="3">
         <v>79</v>
       </c>
       <c r="F80" s="4"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:6">
       <c r="A81" s="3">
         <v>80</v>
       </c>
       <c r="F81" s="4"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:6">
       <c r="A82" s="3">
         <v>81</v>
       </c>
       <c r="F82" s="4"/>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:6">
       <c r="A83" s="3">
         <v>82</v>
       </c>
       <c r="F83" s="4"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:6">
       <c r="A84" s="3">
         <v>83</v>
       </c>
       <c r="F84" s="4"/>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:6">
       <c r="A85" s="3">
         <v>84</v>
       </c>
       <c r="F85" s="4"/>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:6">
       <c r="A86" s="3">
         <v>85</v>
       </c>
       <c r="F86" s="4"/>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:6">
       <c r="A87" s="3">
         <v>86</v>
       </c>
       <c r="F87" s="4"/>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:6">
       <c r="A88" s="3">
         <v>87</v>
       </c>
       <c r="F88" s="4"/>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:6">
       <c r="A89" s="3">
         <v>88</v>
       </c>
       <c r="F89" s="4"/>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:6">
       <c r="A90" s="3">
         <v>89</v>
       </c>
       <c r="F90" s="4"/>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:6">
       <c r="A91" s="3">
         <v>90</v>
       </c>
       <c r="F91" s="4"/>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:6">
       <c r="A92" s="3">
         <v>91</v>
       </c>
       <c r="F92" s="4"/>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:6">
       <c r="A93" s="3">
         <v>92</v>
       </c>
       <c r="F93" s="4"/>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:6">
       <c r="A94" s="3">
         <v>93</v>
       </c>
       <c r="F94" s="4"/>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:6">
       <c r="A95" s="3">
         <v>94</v>
       </c>
       <c r="F95" s="4"/>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:6">
       <c r="A96" s="3">
         <v>95</v>
       </c>
       <c r="F96" s="4"/>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:6">
       <c r="A97" s="3">
         <v>96</v>
       </c>
       <c r="F97" s="4"/>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:6">
       <c r="A98" s="3">
         <v>97</v>
       </c>
       <c r="F98" s="4"/>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:6">
       <c r="A99" s="3">
         <v>98</v>
       </c>
       <c r="F99" s="4"/>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:6">
       <c r="A100" s="3">
         <v>99</v>
       </c>
       <c r="F100" s="4"/>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:6">
       <c r="F101" s="4"/>
     </row>
   </sheetData>
@@ -2275,26 +2345,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f2c92a4b-fdf1-4091-a3b5-730e0262f810">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ed40aa6c-982d-4d5a-abf0-52239ff24e20" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBBF1B2C966E054EA174FC74AC82655E" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c104540bbb065d28aa5cf3f4eef6ea0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f2c92a4b-fdf1-4091-a3b5-730e0262f810" xmlns:ns3="ed40aa6c-982d-4d5a-abf0-52239ff24e20" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2f96469c0e5fa76c57eb88cc3ffabdde" ns2:_="" ns3:_="">
     <xsd:import namespace="f2c92a4b-fdf1-4091-a3b5-730e0262f810"/>
@@ -2489,10 +2539,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f2c92a4b-fdf1-4091-a3b5-730e0262f810">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ed40aa6c-982d-4d5a-abf0-52239ff24e20" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{805F7998-CA6B-4F3D-A9AA-6D44C530CD4E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CCAA9D4-BAE8-42AB-9344-279723EC1018}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f2c92a4b-fdf1-4091-a3b5-730e0262f810"/>
+    <ds:schemaRef ds:uri="ed40aa6c-982d-4d5a-abf0-52239ff24e20"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2509,20 +2590,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CCAA9D4-BAE8-42AB-9344-279723EC1018}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{805F7998-CA6B-4F3D-A9AA-6D44C530CD4E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f2c92a4b-fdf1-4091-a3b5-730e0262f810"/>
-    <ds:schemaRef ds:uri="ed40aa6c-982d-4d5a-abf0-52239ff24e20"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>